<commit_message>
Regenerate delivery zone indicator (2026-10-30)
</commit_message>
<xml_diff>
--- a/data/delivery_zones_2026.xlsx
+++ b/data/delivery_zones_2026.xlsx
@@ -454,7 +454,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
     </row>
@@ -474,7 +474,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
     </row>
@@ -494,7 +494,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
     </row>
@@ -534,7 +534,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
     </row>
@@ -574,7 +574,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
     </row>
@@ -594,7 +594,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
     </row>
@@ -614,7 +614,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
     </row>
@@ -634,7 +634,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
     </row>
@@ -654,7 +654,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
     </row>
@@ -674,7 +674,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
     </row>
@@ -694,7 +694,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
     </row>
@@ -754,7 +754,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
     </row>
@@ -774,7 +774,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
     </row>
@@ -794,7 +794,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
     </row>
@@ -814,7 +814,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
     </row>
@@ -854,7 +854,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
     </row>
@@ -894,7 +894,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
     </row>
@@ -954,7 +954,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
     </row>
@@ -1234,7 +1234,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
     </row>
@@ -1254,7 +1254,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
     </row>
@@ -1294,7 +1294,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
     </row>
@@ -1314,7 +1314,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
     </row>
@@ -1374,7 +1374,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
     </row>
@@ -1454,7 +1454,7 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
     </row>
@@ -18554,7 +18554,7 @@
       </c>
       <c r="D907" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
     </row>

</xml_diff>